<commit_message>
Atualiza painel com gráficos por mercado e evolução mensal
</commit_message>
<xml_diff>
--- a/Investimento_Modelo_Capital_Por_Estrategia.xlsx
+++ b/Investimento_Modelo_Capital_Por_Estrategia.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\Planilha de Investimento\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2147DF41-7762-4B0C-815E-1E1AEA0DE500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B10E3CD-E48D-4643-A66F-3B13C92A3F7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lançamentos" sheetId="1" r:id="rId1"/>
@@ -121,11 +121,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -428,8 +429,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
+    <col min="4" max="4" width="26.28515625" customWidth="1"/>
+    <col min="5" max="5" width="30.42578125" customWidth="1"/>
+    <col min="6" max="6" width="22.42578125" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="8" max="8" width="20.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -455,6 +466,156 @@
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>45748</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>45749</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>45750</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>45751</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>45752</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>45753</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>45754</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>45755</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>45756</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>45757</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>45758</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>45759</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>45760</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>45761</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>45762</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>45763</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>45764</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
+        <v>45765</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <v>45766</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <v>45767</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
+        <v>45768</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
+        <v>45769</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2">
+        <v>45770</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2">
+        <v>45771</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2">
+        <v>45772</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2">
+        <v>45773</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2">
+        <v>45774</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2">
+        <v>45775</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
+        <v>45776</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <v>45777</v>
       </c>
     </row>
   </sheetData>
@@ -466,6 +627,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="3" max="4" width="21.42578125" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -486,7 +653,7 @@
         <v>11</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -494,7 +661,7 @@
         <v>12</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -502,7 +669,7 @@
         <v>13</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -510,7 +677,7 @@
         <v>14</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>